<commit_message>
Added new book: este es un libro by prueba in Nini's library
</commit_message>
<xml_diff>
--- a/data/nini/Biblioteca.xlsx
+++ b/data/nini/Biblioteca.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C313"/>
+  <dimension ref="A1:C314"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5669,6 +5669,23 @@
         </is>
       </c>
     </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>este es un libro</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>prueba</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>otr</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Deleted book: este es un libro from Nini's library
</commit_message>
<xml_diff>
--- a/data/nini/Biblioteca.xlsx
+++ b/data/nini/Biblioteca.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C314"/>
+  <dimension ref="A1:C313"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5669,23 +5669,6 @@
         </is>
       </c>
     </row>
-    <row r="314">
-      <c r="A314" t="inlineStr">
-        <is>
-          <t>este es un libro</t>
-        </is>
-      </c>
-      <c r="B314" t="inlineStr">
-        <is>
-          <t>prueba</t>
-        </is>
-      </c>
-      <c r="C314" t="inlineStr">
-        <is>
-          <t>otr</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Moved book 'La mujer zorro y el doctor Shimamura' from wishlist to biblioteca
</commit_message>
<xml_diff>
--- a/data/nini/Biblioteca.xlsx
+++ b/data/nini/Biblioteca.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C313"/>
+  <dimension ref="A1:C314"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5669,6 +5669,23 @@
         </is>
       </c>
     </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>La mujer zorro y el doctor Shimamura</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>Christine Wunnicke</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>Impedimenta</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Deleted book: La mujer zorro y el doctor Shimamura from Nini's library
</commit_message>
<xml_diff>
--- a/data/nini/Biblioteca.xlsx
+++ b/data/nini/Biblioteca.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C315"/>
+  <dimension ref="A1:C314"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5686,23 +5686,6 @@
         </is>
       </c>
     </row>
-    <row r="315">
-      <c r="A315" t="inlineStr">
-        <is>
-          <t>La mujer zorro y el doctor Shimamura</t>
-        </is>
-      </c>
-      <c r="B315" t="inlineStr">
-        <is>
-          <t>Christine Wunnicke</t>
-        </is>
-      </c>
-      <c r="C315" t="inlineStr">
-        <is>
-          <t>Impedimenta</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Moved book 'Hamnet' from wishlist to biblioteca
</commit_message>
<xml_diff>
--- a/data/nini/Biblioteca.xlsx
+++ b/data/nini/Biblioteca.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H328"/>
+  <dimension ref="A1:H329"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7580,6 +7580,28 @@
       <c r="G328" t="inlineStr"/>
       <c r="H328" t="inlineStr"/>
     </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>Hamnet</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>Maggie O'Farrell</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>Libros del Asteroide</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr"/>
+      <c r="E329" t="inlineStr"/>
+      <c r="F329" t="inlineStr"/>
+      <c r="G329" t="inlineStr"/>
+      <c r="H329" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Added new book: Cuentos Ilustres by Saki in Nini's library
</commit_message>
<xml_diff>
--- a/data/nini/Biblioteca.xlsx
+++ b/data/nini/Biblioteca.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H329"/>
+  <dimension ref="A1:H330"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7602,6 +7602,28 @@
       <c r="G329" t="inlineStr"/>
       <c r="H329" t="inlineStr"/>
     </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>Cuentos Ilustres</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>Saki</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>Alma</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr"/>
+      <c r="E330" t="inlineStr"/>
+      <c r="F330" t="inlineStr"/>
+      <c r="G330" t="inlineStr"/>
+      <c r="H330" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Moved book 'El mundo de ayer' from wishlist to biblioteca
</commit_message>
<xml_diff>
--- a/data/nini/Biblioteca.xlsx
+++ b/data/nini/Biblioteca.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H330"/>
+  <dimension ref="A1:H331"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7624,6 +7624,28 @@
       <c r="G330" t="inlineStr"/>
       <c r="H330" t="inlineStr"/>
     </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>El mundo de ayer</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>Stefan Zweig</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>Alma</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr"/>
+      <c r="E331" t="inlineStr"/>
+      <c r="F331" t="inlineStr"/>
+      <c r="G331" t="inlineStr"/>
+      <c r="H331" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Moved book 'Siddhartha' from wishlist to biblioteca
</commit_message>
<xml_diff>
--- a/data/nini/Biblioteca.xlsx
+++ b/data/nini/Biblioteca.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H331"/>
+  <dimension ref="A1:H332"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7646,6 +7646,28 @@
       <c r="G331" t="inlineStr"/>
       <c r="H331" t="inlineStr"/>
     </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>Siddhartha</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>Herman Hesse</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>Debolsillo Edición Especial en Tapa Dura</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr"/>
+      <c r="E332" t="inlineStr"/>
+      <c r="F332" t="inlineStr"/>
+      <c r="G332" t="inlineStr"/>
+      <c r="H332" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Added new book: Crimen y castigo by Fiódor Dostoyevski in Nini's library
</commit_message>
<xml_diff>
--- a/data/nini/Biblioteca.xlsx
+++ b/data/nini/Biblioteca.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H332"/>
+  <dimension ref="A1:H333"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7668,6 +7668,28 @@
       <c r="G332" t="inlineStr"/>
       <c r="H332" t="inlineStr"/>
     </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>Crimen y castigo</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>Fiódor Dostoyevski</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>Alma</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr"/>
+      <c r="E333" t="inlineStr"/>
+      <c r="F333" t="inlineStr"/>
+      <c r="G333" t="inlineStr"/>
+      <c r="H333" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Added new book: Adiós a las armas by Ernest Hemingway in Nini's library
</commit_message>
<xml_diff>
--- a/data/nini/Biblioteca.xlsx
+++ b/data/nini/Biblioteca.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H333"/>
+  <dimension ref="A1:H334"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7690,6 +7690,28 @@
       <c r="G333" t="inlineStr"/>
       <c r="H333" t="inlineStr"/>
     </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>Adiós a las armas</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>Ernest Hemingway</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>Alma</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr"/>
+      <c r="E334" t="inlineStr"/>
+      <c r="F334" t="inlineStr"/>
+      <c r="G334" t="inlineStr"/>
+      <c r="H334" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Added new book: La chica que vive al final del camino by Laird Koenig in Nini's library
</commit_message>
<xml_diff>
--- a/data/nini/Biblioteca.xlsx
+++ b/data/nini/Biblioteca.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H334"/>
+  <dimension ref="A1:H335"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7712,6 +7712,28 @@
       <c r="G334" t="inlineStr"/>
       <c r="H334" t="inlineStr"/>
     </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>La chica que vive al final del camino</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>Laird Koenig</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>Impedimenta</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr"/>
+      <c r="E335" t="inlineStr"/>
+      <c r="F335" t="inlineStr"/>
+      <c r="G335" t="inlineStr"/>
+      <c r="H335" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Added new book: Los muertos no eran tantos by Jenny Valencia in Nini's library
</commit_message>
<xml_diff>
--- a/data/nini/Biblioteca.xlsx
+++ b/data/nini/Biblioteca.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H335"/>
+  <dimension ref="A1:H336"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7734,6 +7734,28 @@
       <c r="G335" t="inlineStr"/>
       <c r="H335" t="inlineStr"/>
     </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>Los muertos no eran tantos</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>Jenny Valencia</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>Angosta</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr"/>
+      <c r="E336" t="inlineStr"/>
+      <c r="F336" t="inlineStr"/>
+      <c r="G336" t="inlineStr"/>
+      <c r="H336" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Added new book: Segunda casa by Rachel Cusk in Nini's library
</commit_message>
<xml_diff>
--- a/data/nini/Biblioteca.xlsx
+++ b/data/nini/Biblioteca.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H336"/>
+  <dimension ref="A1:H337"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7756,6 +7756,28 @@
       <c r="G336" t="inlineStr"/>
       <c r="H336" t="inlineStr"/>
     </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>Segunda casa</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>Rachel Cusk</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>Libros del Asteroide</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr"/>
+      <c r="E337" t="inlineStr"/>
+      <c r="F337" t="inlineStr"/>
+      <c r="G337" t="inlineStr"/>
+      <c r="H337" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Added new book: Cuentos de amor de locura y de muerte by Horacio Quiroga in Nini's library
</commit_message>
<xml_diff>
--- a/data/nini/Biblioteca.xlsx
+++ b/data/nini/Biblioteca.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H337"/>
+  <dimension ref="A1:H338"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7778,6 +7778,28 @@
       <c r="G337" t="inlineStr"/>
       <c r="H337" t="inlineStr"/>
     </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>Cuentos de amor de locura y de muerte</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>Horacio Quiroga</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>Alma</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr"/>
+      <c r="E338" t="inlineStr"/>
+      <c r="F338" t="inlineStr"/>
+      <c r="G338" t="inlineStr"/>
+      <c r="H338" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Added new book: Tránsito by Rachel Cusk in Nini's library
</commit_message>
<xml_diff>
--- a/data/nini/Biblioteca.xlsx
+++ b/data/nini/Biblioteca.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H338"/>
+  <dimension ref="A1:H339"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7800,6 +7800,28 @@
       <c r="G338" t="inlineStr"/>
       <c r="H338" t="inlineStr"/>
     </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>Tránsito</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>Rachel Cusk</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>Libros del Asteroide</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr"/>
+      <c r="E339" t="inlineStr"/>
+      <c r="F339" t="inlineStr"/>
+      <c r="G339" t="inlineStr"/>
+      <c r="H339" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Added new book: La librería by Penelope Fitzgerald in Nini's library
</commit_message>
<xml_diff>
--- a/data/nini/Biblioteca.xlsx
+++ b/data/nini/Biblioteca.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H339"/>
+  <dimension ref="A1:H340"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7822,6 +7822,28 @@
       <c r="G339" t="inlineStr"/>
       <c r="H339" t="inlineStr"/>
     </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>La librería</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>Penelope Fitzgerald</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>Impedimenta</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr"/>
+      <c r="E340" t="inlineStr"/>
+      <c r="F340" t="inlineStr"/>
+      <c r="G340" t="inlineStr"/>
+      <c r="H340" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Added new book: Rojo y negro by Stendhal in Nini's library
</commit_message>
<xml_diff>
--- a/data/nini/Biblioteca.xlsx
+++ b/data/nini/Biblioteca.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H340"/>
+  <dimension ref="A1:H341"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7844,6 +7844,28 @@
       <c r="G340" t="inlineStr"/>
       <c r="H340" t="inlineStr"/>
     </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>Rojo y negro</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>Stendhal</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>Alma</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr"/>
+      <c r="E341" t="inlineStr"/>
+      <c r="F341" t="inlineStr"/>
+      <c r="G341" t="inlineStr"/>
+      <c r="H341" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Added new book: Bajo el ojo del gran pájaro by Hiromi Kawakami in Nini's library
</commit_message>
<xml_diff>
--- a/data/nini/Biblioteca.xlsx
+++ b/data/nini/Biblioteca.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H341"/>
+  <dimension ref="A1:H342"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7866,6 +7866,28 @@
       <c r="G341" t="inlineStr"/>
       <c r="H341" t="inlineStr"/>
     </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>Bajo el ojo del gran pájaro</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>Hiromi Kawakami</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>Alfaguara</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr"/>
+      <c r="E342" t="inlineStr"/>
+      <c r="F342" t="inlineStr"/>
+      <c r="G342" t="inlineStr"/>
+      <c r="H342" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Added new book: El santo del monte Koya y otros relatos by Izumi Kyōka in Nini's library
</commit_message>
<xml_diff>
--- a/data/nini/Biblioteca.xlsx
+++ b/data/nini/Biblioteca.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H342"/>
+  <dimension ref="A1:H343"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7888,6 +7888,28 @@
       <c r="G342" t="inlineStr"/>
       <c r="H342" t="inlineStr"/>
     </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>El santo del monte Koya y otros relatos</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>Izumi Kyōka</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>Satori</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr"/>
+      <c r="E343" t="inlineStr"/>
+      <c r="F343" t="inlineStr"/>
+      <c r="G343" t="inlineStr"/>
+      <c r="H343" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Added new book: Matar a un ruiseñor by Harper Lee in Nini's library
</commit_message>
<xml_diff>
--- a/data/nini/Biblioteca.xlsx
+++ b/data/nini/Biblioteca.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H344"/>
+  <dimension ref="A1:H345"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7932,6 +7932,28 @@
       <c r="G344" t="inlineStr"/>
       <c r="H344" t="inlineStr"/>
     </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>Matar a un ruiseñor</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>Harper Lee</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>Harper Collins</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr"/>
+      <c r="E345" t="inlineStr"/>
+      <c r="F345" t="inlineStr"/>
+      <c r="G345" t="inlineStr"/>
+      <c r="H345" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Added new book: El año del hambre by Aki Ollikainen in Nini's library
</commit_message>
<xml_diff>
--- a/data/nini/Biblioteca.xlsx
+++ b/data/nini/Biblioteca.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H345"/>
+  <dimension ref="A1:H346"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7954,6 +7954,28 @@
       <c r="G345" t="inlineStr"/>
       <c r="H345" t="inlineStr"/>
     </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>El año del hambre</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>Aki Ollikainen</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>Libros del Asteroide</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr"/>
+      <c r="E346" t="inlineStr"/>
+      <c r="F346" t="inlineStr"/>
+      <c r="G346" t="inlineStr"/>
+      <c r="H346" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Deleted book: El santo del monte Koya y otros relatos from Nini's library
</commit_message>
<xml_diff>
--- a/data/nini/Biblioteca.xlsx
+++ b/data/nini/Biblioteca.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H346"/>
+  <dimension ref="A1:H345"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7913,17 +7913,17 @@
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>El santo del monte Koya y otros relatos</t>
+          <t>Matar a un ruiseñor</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>Izumi Kyōka</t>
+          <t>Harper Lee</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>Satori</t>
+          <t>Harper Collins</t>
         </is>
       </c>
       <c r="D344" t="inlineStr"/>
@@ -7935,17 +7935,17 @@
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>Matar a un ruiseñor</t>
+          <t>El año del hambre</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>Harper Lee</t>
+          <t>Aki Ollikainen</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>Harper Collins</t>
+          <t>Libros del Asteroide</t>
         </is>
       </c>
       <c r="D345" t="inlineStr"/>
@@ -7954,28 +7954,6 @@
       <c r="G345" t="inlineStr"/>
       <c r="H345" t="inlineStr"/>
     </row>
-    <row r="346">
-      <c r="A346" t="inlineStr">
-        <is>
-          <t>El año del hambre</t>
-        </is>
-      </c>
-      <c r="B346" t="inlineStr">
-        <is>
-          <t>Aki Ollikainen</t>
-        </is>
-      </c>
-      <c r="C346" t="inlineStr">
-        <is>
-          <t>Libros del Asteroide</t>
-        </is>
-      </c>
-      <c r="D346" t="inlineStr"/>
-      <c r="E346" t="inlineStr"/>
-      <c r="F346" t="inlineStr"/>
-      <c r="G346" t="inlineStr"/>
-      <c r="H346" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Added new book: Moby Dick by Herman Melville in Nini's library
</commit_message>
<xml_diff>
--- a/data/nini/Biblioteca.xlsx
+++ b/data/nini/Biblioteca.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H345"/>
+  <dimension ref="A1:H346"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7954,6 +7954,28 @@
       <c r="G345" t="inlineStr"/>
       <c r="H345" t="inlineStr"/>
     </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>Moby Dick</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>Herman Melville</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>Alma</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr"/>
+      <c r="E346" t="inlineStr"/>
+      <c r="F346" t="inlineStr"/>
+      <c r="G346" t="inlineStr"/>
+      <c r="H346" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Moved book 'To kill a mockingbird' from wishlist to biblioteca
</commit_message>
<xml_diff>
--- a/data/nini/Biblioteca.xlsx
+++ b/data/nini/Biblioteca.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H346"/>
+  <dimension ref="A1:H347"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7976,6 +7976,28 @@
       <c r="G346" t="inlineStr"/>
       <c r="H346" t="inlineStr"/>
     </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>To kill a mockingbird</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>Harper Lee</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>Harper Collins</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr"/>
+      <c r="E347" t="inlineStr"/>
+      <c r="F347" t="inlineStr"/>
+      <c r="G347" t="inlineStr"/>
+      <c r="H347" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Moved book 'Cartago' from wishlist to biblioteca
</commit_message>
<xml_diff>
--- a/data/nini/Biblioteca.xlsx
+++ b/data/nini/Biblioteca.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H347"/>
+  <dimension ref="A1:H348"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7998,6 +7998,28 @@
       <c r="G347" t="inlineStr"/>
       <c r="H347" t="inlineStr"/>
     </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>Cartago</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>Daniel Cristancho</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>Angosta</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr"/>
+      <c r="E348" t="inlineStr"/>
+      <c r="F348" t="inlineStr"/>
+      <c r="G348" t="inlineStr"/>
+      <c r="H348" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Moved book 'La aventura de Miguel Littín clandestino en Chile' from wishlist to biblioteca
</commit_message>
<xml_diff>
--- a/data/nini/Biblioteca.xlsx
+++ b/data/nini/Biblioteca.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H348"/>
+  <dimension ref="A1:H349"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8020,6 +8020,24 @@
       <c r="G348" t="inlineStr"/>
       <c r="H348" t="inlineStr"/>
     </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>La aventura de Miguel Littín clandestino en Chile</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>Gabriel García Márquez</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr"/>
+      <c r="D349" t="inlineStr"/>
+      <c r="E349" t="inlineStr"/>
+      <c r="F349" t="inlineStr"/>
+      <c r="G349" t="inlineStr"/>
+      <c r="H349" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Added new book: El gran Gatsby by Francis Scott Fitzgerald in Nini's library
</commit_message>
<xml_diff>
--- a/data/nini/Biblioteca.xlsx
+++ b/data/nini/Biblioteca.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H349"/>
+  <dimension ref="A1:H350"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8038,6 +8038,28 @@
       <c r="G349" t="inlineStr"/>
       <c r="H349" t="inlineStr"/>
     </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>El gran Gatsby</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>Francis Scott Fitzgerald</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>DeBolsillo</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr"/>
+      <c r="E350" t="inlineStr"/>
+      <c r="F350" t="inlineStr"/>
+      <c r="G350" t="inlineStr"/>
+      <c r="H350" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Moved book '1984' from wishlist to biblioteca
</commit_message>
<xml_diff>
--- a/data/nini/Biblioteca.xlsx
+++ b/data/nini/Biblioteca.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H350"/>
+  <dimension ref="A1:H351"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8060,6 +8060,26 @@
       <c r="G350" t="inlineStr"/>
       <c r="H350" t="inlineStr"/>
     </row>
+    <row r="351">
+      <c r="A351" t="n">
+        <v>1984</v>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>George Orwell</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>Debolsillo Edición Especial en Tapa Dura</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr"/>
+      <c r="E351" t="inlineStr"/>
+      <c r="F351" t="inlineStr"/>
+      <c r="G351" t="inlineStr"/>
+      <c r="H351" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated book: La aventura de Miguel Littín clandestino en Chile by Gabriel García Márquez in Nini's library
</commit_message>
<xml_diff>
--- a/data/nini/Biblioteca.xlsx
+++ b/data/nini/Biblioteca.xlsx
@@ -8031,7 +8031,11 @@
           <t>Gabriel García Márquez</t>
         </is>
       </c>
-      <c r="C349" t="inlineStr"/>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>Debolsillo</t>
+        </is>
+      </c>
       <c r="D349" t="inlineStr"/>
       <c r="E349" t="inlineStr"/>
       <c r="F349" t="inlineStr"/>

</xml_diff>

<commit_message>
Updated book: 1984 by George Orwell in Nini's library
</commit_message>
<xml_diff>
--- a/data/nini/Biblioteca.xlsx
+++ b/data/nini/Biblioteca.xlsx
@@ -8065,8 +8065,10 @@
       <c r="H350" t="inlineStr"/>
     </row>
     <row r="351">
-      <c r="A351" t="n">
-        <v>1984</v>
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>1984</t>
+        </is>
       </c>
       <c r="B351" t="inlineStr">
         <is>
@@ -8075,7 +8077,7 @@
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>Debolsillo Edición Especial en Tapa Dura</t>
+          <t>DeBolsillo</t>
         </is>
       </c>
       <c r="D351" t="inlineStr"/>

</xml_diff>

<commit_message>
Added new book: La tormenta de nieve by Lev Tolstói in Nini's library
</commit_message>
<xml_diff>
--- a/data/nini/Biblioteca.xlsx
+++ b/data/nini/Biblioteca.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H351"/>
+  <dimension ref="A1:H352"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8086,6 +8086,28 @@
       <c r="G351" t="inlineStr"/>
       <c r="H351" t="inlineStr"/>
     </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>La tormenta de nieve</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>Lev Tolstói</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>Alma</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr"/>
+      <c r="E352" t="inlineStr"/>
+      <c r="F352" t="inlineStr"/>
+      <c r="G352" t="inlineStr"/>
+      <c r="H352" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Added new book: Las niñas aprendemos en silencio by Catalina Gallo in Nini's library
</commit_message>
<xml_diff>
--- a/data/nini/Biblioteca.xlsx
+++ b/data/nini/Biblioteca.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H352"/>
+  <dimension ref="A1:H353"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8108,6 +8108,28 @@
       <c r="G352" t="inlineStr"/>
       <c r="H352" t="inlineStr"/>
     </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>Las niñas aprendemos en silencio</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>Catalina Gallo</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>Laguna libros</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr"/>
+      <c r="E353" t="inlineStr"/>
+      <c r="F353" t="inlineStr"/>
+      <c r="G353" t="inlineStr"/>
+      <c r="H353" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Added new book: En ninguna parte by Bae Suah in Nini's library
</commit_message>
<xml_diff>
--- a/data/nini/Biblioteca.xlsx
+++ b/data/nini/Biblioteca.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H353"/>
+  <dimension ref="A1:H354"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8130,6 +8130,28 @@
       <c r="G353" t="inlineStr"/>
       <c r="H353" t="inlineStr"/>
     </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>En ninguna parte</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>Bae Suah</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>Shiro</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr"/>
+      <c r="E354" t="inlineStr"/>
+      <c r="F354" t="inlineStr"/>
+      <c r="G354" t="inlineStr"/>
+      <c r="H354" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Added new book: Ya nadie escribe cartas by Jang Eun-jin in Nini's library
</commit_message>
<xml_diff>
--- a/data/nini/Biblioteca.xlsx
+++ b/data/nini/Biblioteca.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H354"/>
+  <dimension ref="A1:H355"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8152,6 +8152,28 @@
       <c r="G354" t="inlineStr"/>
       <c r="H354" t="inlineStr"/>
     </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>Ya nadie escribe cartas</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>Jang Eun-jin</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>Shiro</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr"/>
+      <c r="E355" t="inlineStr"/>
+      <c r="F355" t="inlineStr"/>
+      <c r="G355" t="inlineStr"/>
+      <c r="H355" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Added new book: Nada dentro by Asako Otani in Nini's library
</commit_message>
<xml_diff>
--- a/data/nini/Biblioteca.xlsx
+++ b/data/nini/Biblioteca.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H355"/>
+  <dimension ref="A1:H356"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8174,6 +8174,28 @@
       <c r="G355" t="inlineStr"/>
       <c r="H355" t="inlineStr"/>
     </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>Nada dentro</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>Asako Otani</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>Shiro</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr"/>
+      <c r="E356" t="inlineStr"/>
+      <c r="F356" t="inlineStr"/>
+      <c r="G356" t="inlineStr"/>
+      <c r="H356" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Added new book: Dradradragón by Park Min-gyu in Nini's library
</commit_message>
<xml_diff>
--- a/data/nini/Biblioteca.xlsx
+++ b/data/nini/Biblioteca.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H356"/>
+  <dimension ref="A1:H357"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8196,6 +8196,28 @@
       <c r="G356" t="inlineStr"/>
       <c r="H356" t="inlineStr"/>
     </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>Dradradragón</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>Park Min-gyu</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>Shiro</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr"/>
+      <c r="E357" t="inlineStr"/>
+      <c r="F357" t="inlineStr"/>
+      <c r="G357" t="inlineStr"/>
+      <c r="H357" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>